<commit_message>
fixed xase study and skills
</commit_message>
<xml_diff>
--- a/skillsprogressiontable_18-8-25.xlsx
+++ b/skillsprogressiontable_18-8-25.xlsx
@@ -1,19 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gla-my.sharepoint.com/personal/helena_paterson_glasgow_ac_uk/Documents/SOTL/AI in assessment chapter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gla-my.sharepoint.com/personal/helena_paterson_glasgow_ac_uk/Documents/Documents/assessmentai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="240" documentId="13_ncr:1_{1F80AE8C-8A3C-FD4D-A675-5315F92D8B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9EC600C-6EAB-C648-A404-287034DCA6CC}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="13_ncr:1_{1F80AE8C-8A3C-FD4D-A675-5315F92D8B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A550009A-A8E3-42AF-A887-74EBB73AB074}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28320" windowHeight="16840" xr2:uid="{3FD2D535-207D-B548-9150-2445C489AFDF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3FD2D535-207D-B548-9150-2445C489AFDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="200">
   <si>
     <t>1st Year - Laboratory Practical</t>
   </si>
@@ -775,23 +779,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -807,6 +802,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1143,76 +1147,76 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{377F8B1A-6932-EE44-BDFE-5FB345D0E742}">
   <dimension ref="A1:Y14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.6640625" customWidth="1"/>
-    <col min="2" max="2" width="2.83203125" customWidth="1"/>
+    <col min="1" max="1" width="37.69921875" customWidth="1"/>
+    <col min="2" max="2" width="2.796875" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="4" width="58.1640625" customWidth="1"/>
-    <col min="5" max="5" width="43.6640625" customWidth="1"/>
-    <col min="6" max="6" width="43.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="28.1640625" customWidth="1"/>
-    <col min="8" max="8" width="2.6640625" customWidth="1"/>
-    <col min="9" max="9" width="42.83203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="58.19921875" customWidth="1"/>
+    <col min="5" max="5" width="43.69921875" customWidth="1"/>
+    <col min="6" max="6" width="43.69921875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="28.19921875" customWidth="1"/>
+    <col min="8" max="8" width="2.69921875" customWidth="1"/>
+    <col min="9" max="9" width="42.796875" style="3" customWidth="1"/>
     <col min="10" max="12" width="61" customWidth="1"/>
     <col min="13" max="13" width="36.5" customWidth="1"/>
-    <col min="14" max="14" width="4.83203125" customWidth="1"/>
-    <col min="15" max="15" width="40.1640625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="47.1640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="4.796875" customWidth="1"/>
+    <col min="15" max="15" width="40.19921875" style="3" customWidth="1"/>
+    <col min="16" max="16" width="47.19921875" style="3" customWidth="1"/>
     <col min="17" max="17" width="36.5" style="3" customWidth="1"/>
-    <col min="18" max="18" width="43.83203125" style="3" customWidth="1"/>
-    <col min="19" max="19" width="32.83203125" style="3" customWidth="1"/>
-    <col min="20" max="20" width="3.83203125" style="3" customWidth="1"/>
-    <col min="21" max="21" width="31.33203125" customWidth="1"/>
-    <col min="22" max="22" width="51.33203125" customWidth="1"/>
+    <col min="18" max="18" width="43.796875" style="3" customWidth="1"/>
+    <col min="19" max="19" width="32.796875" style="3" customWidth="1"/>
+    <col min="20" max="20" width="3.796875" style="3" customWidth="1"/>
+    <col min="21" max="21" width="31.296875" customWidth="1"/>
+    <col min="22" max="22" width="51.296875" customWidth="1"/>
     <col min="23" max="24" width="43.5" customWidth="1"/>
-    <col min="25" max="25" width="38.6640625" customWidth="1"/>
+    <col min="25" max="25" width="38.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="109" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:25" ht="109.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="C2" s="24" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="C2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="O2" s="18" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="O2" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-      <c r="S2" s="16"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="15" t="s">
+      <c r="U2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="X2" s="16"/>
-      <c r="Y2" s="16"/>
-    </row>
-    <row r="3" spans="1:25" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+    </row>
+    <row r="3" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1278,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:25" s="10" customFormat="1" ht="238" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" s="10" customFormat="1" ht="218.4" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
@@ -1345,7 +1349,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:25" s="10" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" s="10" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>17</v>
       </c>
@@ -1412,7 +1416,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="12" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" s="12" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>23</v>
       </c>
@@ -1479,7 +1483,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:25" s="10" customFormat="1" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" s="10" customFormat="1" ht="135" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>31</v>
       </c>
@@ -1546,7 +1550,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:25" s="10" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" s="10" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>36</v>
       </c>
@@ -1612,7 +1616,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:25" s="10" customFormat="1" ht="102" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" s="10" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>43</v>
       </c>
@@ -1679,7 +1683,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="10" customFormat="1" ht="136" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" s="10" customFormat="1" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>50</v>
       </c>
@@ -1746,7 +1750,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:25" s="10" customFormat="1" ht="136" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" s="10" customFormat="1" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>60</v>
       </c>
@@ -1813,7 +1817,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:25" s="10" customFormat="1" ht="145" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:25" s="10" customFormat="1" ht="145.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>67</v>
       </c>
@@ -1879,14 +1883,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:25" s="10" customFormat="1" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" s="10" customFormat="1" ht="46.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>72</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="21"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="17"/>
       <c r="F13" s="17"/>
       <c r="G13" s="17"/>
@@ -1927,14 +1931,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="10" customFormat="1" ht="175" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" s="10" customFormat="1" ht="175.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>80</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="21"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
@@ -1967,6 +1971,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="U2:Y2"/>
+    <mergeCell ref="U13:U14"/>
+    <mergeCell ref="V13:V14"/>
+    <mergeCell ref="W13:W14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="P13:P14"/>
+    <mergeCell ref="Q13:Q14"/>
+    <mergeCell ref="S13:S14"/>
+    <mergeCell ref="O2:S2"/>
+    <mergeCell ref="Y13:Y14"/>
+    <mergeCell ref="R13:R14"/>
+    <mergeCell ref="X13:X14"/>
     <mergeCell ref="I2:M2"/>
     <mergeCell ref="D12:D14"/>
     <mergeCell ref="E12:E14"/>
@@ -1979,18 +1995,931 @@
     <mergeCell ref="M12:M13"/>
     <mergeCell ref="F12:F14"/>
     <mergeCell ref="L12:L13"/>
-    <mergeCell ref="U2:Y2"/>
-    <mergeCell ref="U13:U14"/>
-    <mergeCell ref="V13:V14"/>
-    <mergeCell ref="W13:W14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="P13:P14"/>
-    <mergeCell ref="Q13:Q14"/>
-    <mergeCell ref="S13:S14"/>
-    <mergeCell ref="O2:S2"/>
-    <mergeCell ref="Y13:Y14"/>
-    <mergeCell ref="R13:R14"/>
-    <mergeCell ref="X13:X14"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DF191D-B10F-45DD-8503-881AE98A0BBC}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="358.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="327.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="18"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="18"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="E11:E13"/>
+    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="G11:G13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54C8F22E-2A94-4A05-B7C9-7F43B897C7B9}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+    </row>
+    <row r="2" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="390" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="327.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="280.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="358.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+    </row>
+    <row r="13" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68638826-F848-4768-853A-C2071472C7C7}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+    </row>
+    <row r="2" spans="1:5" ht="78" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="312" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FC72B7E-82C0-4C77-9312-B1FE6AC66428}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+    </row>
+    <row r="2" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="327.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>